<commit_message>
WP-B research: fact-check corrections and PDF export
Fix deal years (Insilico-Lilly and Genesis-Incyte are 2026), PostEra's
NIH grant (consortium, not PostEra alone), Stoked seed currency, and
mark unverified prices. Add Iambic-Takeda, print styles and a PDF.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBTPhzVbMdymwAH5WBjFho
</commit_message>
<xml_diff>
--- a/research/stoked-bio-wpb/WP-B_GenChem_Competitor_Database.xlsx
+++ b/research/stoked-bio-wpb/WP-B_GenChem_Competitor_Database.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Competitors'!$A$1:$O$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pricing benchmarks'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal comps'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal comps'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Excluded (biologics)'!$A$1:$B$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -651,11 +651,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>C$2.5M seed (closed May 2026; angel-led, oversubscribed, 99% Ontario investors)</t>
+          <t>$2.5M seed (announced 1 May 2026; angel-led with insiders, oversubscribed, 99% from Ontario; currency not stated, likely CAD)</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>South San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -793,15 +793,15 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>$24M Series A (Jan 2022, Clermont Group); $68M NIH grant (2022, antivirals)</t>
+          <t>$24M Series A (Jan 2022, Clermont Group). Also co-leads the NIH-funded ASAP antiviral consortium ($68M initial funding, shared with MSKCC and DNDi)</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Pfizer AI Lab: $13M upfront / $260M (2022); expanded Jan 2025 with $12M upfront; total Pfizer value reported ~$610M</t>
+          <t>Pfizer AI Lab: $13M upfront, up to $260M (Jan 2022); expanded Jan 2025 with a further $12M upfront</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1014,12 +1014,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Lilly up to $2.75B ($115M upfront); SK Biopharm up to $2.5B; ~$10B aggregate headline value</t>
+          <t>Lilly: $115M upfront, up to $2.75B (Mar 2026); SK Biopharm up to $2.5B; ~$10B aggregate headline value</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Rentosertib (TNIK, IPF) entered global Phase 3 Jul 2026. FY2025 revenue $56.2M, of which software only $4.9M; net loss $352M</t>
+          <t>Rentosertib (TNIK, IPF): Phase 3 launched Jul 2026, first patient dosed 9 Sep 2026. FY2025 revenue $56.2M, of which software only $4.9M; net loss $352M</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>$5.5M seed extension (Feb 2025; Nimbus Synergies lead, Merck GHIF)</t>
+          <t>$3.5M seed (2021) + $5.5M seed extension (Feb 2025; Nimbus Synergies lead, Merck GHIF)</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Lundbeck (migraine), Takeda</t>
+          <t>Takeda: up to $1.7B in milestones, 3 targets (Feb 2026); Lundbeck (migraine, 2024)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Incyte: $80M cash + $40M equity, ~$232M milestones/program; Gilead (2024)</t>
+          <t>Incyte expansion (May 2026): $80M cash + $40M equity, up to $232M milestones per program, 5+ targets; Gilead (2024)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Sanofi up to $140M</t>
+          <t>Sanofi up to $140M (Dec 2023; expanded Jul 2026)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>The default budget line a SyntheMol licence would have to displace; entry pricing ~$10K/seat/yr (third-party estimate). Overlaps with Jonathan's comp-chem slide.</t>
+          <t>The default budget line a SyntheMol licence would have to displace. Prices are quote-only (not published). Overlaps with Jonathan's comp-chem slide.</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Same building-block + reaction-template idea as SyntheMol, using transformers, diffusion or GFlowNets; field grew rapidly from mid-2024.</t>
+          <t>Build molecules from building blocks and reaction templates, the same basic idea as SyntheMol, using transformers, diffusion or GFlowNets; the field grew rapidly from mid-2024.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>The core algorithmic idea is now widely replicated and free. SyntheMol's own code is public on GitHub/PyPI.</t>
+          <t>The core idea is now common in academic work, much of it with public code. SyntheMol's own code is also public on GitHub/PyPI.</t>
         </is>
       </c>
       <c r="M21" s="2" t="n">
@@ -2559,22 +2559,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Schrödinger seat licence</t>
+          <t>Schrödinger licence</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>~$10K per seat per year entry (academic from ~$7.5K)</t>
+          <t>Quote-only; not published. One third-party site estimates ~$10K per seat per year</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Third-party estimate (Capterra/IntuitionLabs)</t>
+          <t>Third-party estimate (IntuitionLabs); Schrödinger site shows no prices</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>List price, verify</t>
+          <t>Unverified</t>
         </is>
       </c>
     </row>
@@ -2586,17 +2586,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>From ~$3K per month; annual plan 16% off; also SaaS, on-prem, or 'discovery sprints'</t>
+          <t>Monthly or yearly plans (yearly 16% off); SaaS, on-prem, or 'discovery sprints'. One third-party site says from ~$3K per month</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Third-party estimate + Insilico site</t>
+          <t>Insilico site (plans); third-party (price)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>List price, verify</t>
+          <t>Price unverified</t>
         </is>
       </c>
     </row>
@@ -2652,17 +2652,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>~$400–700 per compound incl. basic assays; 3–4 weeks; &gt;80% success</t>
+          <t>3–4 weeks, &gt;80% success (Enamine). Cost: one forum estimate of ~$400–700 per compound including basic assays</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PostEra forum estimate / Enamine</t>
+          <t>Enamine / BioSolveIT; PostEra forum post</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Cost unverified</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Plus $40M equity; ~$232M/program × 5</t>
+          <t>Plus $40M equity; headline = up to $232M/program × 5 targets</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>AI Lab; expanded 2025 with $12M upfront</t>
+          <t>AI Lab; expanded Jan 2025 with $12M more upfront</t>
         </is>
       </c>
     </row>
@@ -2914,33 +2914,54 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>€1B+; upfront undisclosed</t>
+          <t>€1B+ (≈$1.08B); upfront undisclosed</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Aqemia → Sanofi</t>
+          <t>Iambic → Takeda</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Milestones only; upfront undisclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Aqemia → Sanofi</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n">
         <v>140</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Upfront undisclosed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E9"/>
+  <autoFilter ref="A1:E10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>